<commit_message>
fix: import data and summary view
</commit_message>
<xml_diff>
--- a/example.xlsx
+++ b/example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dane\sidoreka\Desktop\aplikacje\Odpady_komunalne_aplikacja\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Kurs_python+django\odpady_projekt\municipal-pickup-portal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2785B21D-3574-4E37-A11A-603E7C5143AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28FDDC68-12FA-41CD-9737-BCADC892F5E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4290" yWindow="4290" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,12 +20,15 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
   <si>
     <t>Numer MPK</t>
   </si>
@@ -268,7 +271,7 @@
         <charset val="238"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="19" formatCode="yyyy/mm/dd"/>
+      <numFmt numFmtId="164" formatCode="yyyy/mm/dd"/>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
@@ -593,8 +596,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{13142892-4345-4EC7-92E6-B339FE85BCE4}" name="dane" displayName="dane" ref="A1:G4" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8" totalsRowBorderDxfId="7">
-  <autoFilter ref="A1:G4" xr:uid="{13142892-4345-4EC7-92E6-B339FE85BCE4}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{13142892-4345-4EC7-92E6-B339FE85BCE4}" name="dane" displayName="dane" ref="A1:G6" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8" totalsRowBorderDxfId="7">
+  <autoFilter ref="A1:G6" xr:uid="{13142892-4345-4EC7-92E6-B339FE85BCE4}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{3BF945B2-633C-4E97-B38F-69FC9932D3CD}" name="Numer MPK" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{25E88CE6-EB6E-42B3-9A9A-4C038F00339C}" name="Rok" dataDxfId="5"/>
@@ -871,7 +874,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.28515625" customWidth="1"/>
@@ -950,7 +953,7 @@
         <v>46128</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="7">
         <v>6014</v>
       </c>
@@ -971,6 +974,52 @@
       </c>
       <c r="G4" s="9">
         <v>46150</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="7">
+        <v>6014</v>
+      </c>
+      <c r="B5" s="8">
+        <v>2026</v>
+      </c>
+      <c r="C5" s="8">
+        <v>5</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="8">
+        <v>120</v>
+      </c>
+      <c r="F5" s="8">
+        <v>5</v>
+      </c>
+      <c r="G5" s="3">
+        <v>46157</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="7">
+        <v>6013</v>
+      </c>
+      <c r="B6" s="8">
+        <v>2026</v>
+      </c>
+      <c r="C6" s="8">
+        <v>5</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="8">
+        <v>120</v>
+      </c>
+      <c r="F6" s="8">
+        <v>5</v>
+      </c>
+      <c r="G6" s="3">
+        <v>46157</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: start aplication v2
</commit_message>
<xml_diff>
--- a/example.xlsx
+++ b/example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dane\sidoreka\Desktop\aplikacje\Odpady_komunalne_aplikacja\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Kurs_python+django\odpady_projekt\municipal-pickup-portal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2785B21D-3574-4E37-A11A-603E7C5143AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28FDDC68-12FA-41CD-9737-BCADC892F5E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4290" yWindow="4290" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,12 +20,15 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
   <si>
     <t>Numer MPK</t>
   </si>
@@ -268,7 +271,7 @@
         <charset val="238"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="19" formatCode="yyyy/mm/dd"/>
+      <numFmt numFmtId="164" formatCode="yyyy/mm/dd"/>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
@@ -593,8 +596,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{13142892-4345-4EC7-92E6-B339FE85BCE4}" name="dane" displayName="dane" ref="A1:G4" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8" totalsRowBorderDxfId="7">
-  <autoFilter ref="A1:G4" xr:uid="{13142892-4345-4EC7-92E6-B339FE85BCE4}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{13142892-4345-4EC7-92E6-B339FE85BCE4}" name="dane" displayName="dane" ref="A1:G6" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8" totalsRowBorderDxfId="7">
+  <autoFilter ref="A1:G6" xr:uid="{13142892-4345-4EC7-92E6-B339FE85BCE4}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{3BF945B2-633C-4E97-B38F-69FC9932D3CD}" name="Numer MPK" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{25E88CE6-EB6E-42B3-9A9A-4C038F00339C}" name="Rok" dataDxfId="5"/>
@@ -871,7 +874,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.28515625" customWidth="1"/>
@@ -950,7 +953,7 @@
         <v>46128</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="7">
         <v>6014</v>
       </c>
@@ -971,6 +974,52 @@
       </c>
       <c r="G4" s="9">
         <v>46150</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="7">
+        <v>6014</v>
+      </c>
+      <c r="B5" s="8">
+        <v>2026</v>
+      </c>
+      <c r="C5" s="8">
+        <v>5</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="8">
+        <v>120</v>
+      </c>
+      <c r="F5" s="8">
+        <v>5</v>
+      </c>
+      <c r="G5" s="3">
+        <v>46157</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="7">
+        <v>6013</v>
+      </c>
+      <c r="B6" s="8">
+        <v>2026</v>
+      </c>
+      <c r="C6" s="8">
+        <v>5</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="8">
+        <v>120</v>
+      </c>
+      <c r="F6" s="8">
+        <v>5</v>
+      </c>
+      <c r="G6" s="3">
+        <v>46157</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: improvements to page layout, views and forms
</commit_message>
<xml_diff>
--- a/example.xlsx
+++ b/example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Kurs_python+django\odpady_projekt\municipal-pickup-portal\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dane\sidoreka\Desktop\aplikacje\Odpady_komunalne_aplikacja\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28FDDC68-12FA-41CD-9737-BCADC892F5E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{789CAA68-DF29-4237-84F4-5B27CA06874D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4290" yWindow="4290" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3675" yWindow="4245" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,15 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="10">
   <si>
     <t>Numer MPK</t>
   </si>
@@ -271,7 +268,7 @@
         <charset val="238"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="164" formatCode="yyyy/mm/dd"/>
+      <numFmt numFmtId="19" formatCode="yyyy/mm/dd"/>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
@@ -596,8 +593,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{13142892-4345-4EC7-92E6-B339FE85BCE4}" name="dane" displayName="dane" ref="A1:G6" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8" totalsRowBorderDxfId="7">
-  <autoFilter ref="A1:G6" xr:uid="{13142892-4345-4EC7-92E6-B339FE85BCE4}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{13142892-4345-4EC7-92E6-B339FE85BCE4}" name="dane" displayName="dane" ref="A1:G7" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8" totalsRowBorderDxfId="7">
+  <autoFilter ref="A1:G7" xr:uid="{13142892-4345-4EC7-92E6-B339FE85BCE4}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{3BF945B2-633C-4E97-B38F-69FC9932D3CD}" name="Numer MPK" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{25E88CE6-EB6E-42B3-9A9A-4C038F00339C}" name="Rok" dataDxfId="5"/>
@@ -874,7 +871,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.28515625" customWidth="1"/>
@@ -944,7 +941,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="8">
-        <v>240</v>
+        <v>1100</v>
       </c>
       <c r="F3" s="8">
         <v>2</v>
@@ -1019,6 +1016,29 @@
         <v>5</v>
       </c>
       <c r="G6" s="3">
+        <v>46157</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="7">
+        <v>6014</v>
+      </c>
+      <c r="B7" s="8">
+        <v>2026</v>
+      </c>
+      <c r="C7" s="8">
+        <v>3</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="8">
+        <v>1100</v>
+      </c>
+      <c r="F7" s="8">
+        <v>70</v>
+      </c>
+      <c r="G7" s="9">
         <v>46157</v>
       </c>
     </row>

</xml_diff>